<commit_message>
Update the gallery catalogue
</commit_message>
<xml_diff>
--- a/Indus Art Collection - Catalogue.xlsx
+++ b/Indus Art Collection - Catalogue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="219">
   <si>
     <t>Reference (do not edit)</t>
   </si>
@@ -82,16 +82,31 @@
     <t>IAC-007</t>
   </si>
   <si>
+    <t>48 x 84 in</t>
+  </si>
+  <si>
+    <t>IAC-008</t>
+  </si>
+  <si>
+    <t>IAC-009</t>
+  </si>
+  <si>
+    <t>IAC-010</t>
+  </si>
+  <si>
+    <t>IAC-011</t>
+  </si>
+  <si>
     <t>Triptych</t>
   </si>
   <si>
     <t>18 x 60 in each</t>
   </si>
   <si>
-    <t>IAC-008</t>
-  </si>
-  <si>
-    <t>IAC-009</t>
+    <t>IAC-012</t>
+  </si>
+  <si>
+    <t>IAC-013</t>
   </si>
   <si>
     <t>Kandan G</t>
@@ -109,19 +124,40 @@
     <t>2024</t>
   </si>
   <si>
-    <t>IAC-010</t>
-  </si>
-  <si>
-    <t>IAC-011</t>
+    <t>IAC-014</t>
+  </si>
+  <si>
+    <t>IAC-015</t>
   </si>
   <si>
     <t>36 x 60 in / 92 x 153 cm</t>
   </si>
   <si>
-    <t>IAC-012</t>
-  </si>
-  <si>
-    <t>IAC-013</t>
+    <t>IAC-016</t>
+  </si>
+  <si>
+    <t>IAC-017</t>
+  </si>
+  <si>
+    <t>36 x 65 in / 91 x 165 cm</t>
+  </si>
+  <si>
+    <t>IAC-018</t>
+  </si>
+  <si>
+    <t>IAC-019</t>
+  </si>
+  <si>
+    <t>38 x 74 in / 97 x 187 cm</t>
+  </si>
+  <si>
+    <t>IAC-020</t>
+  </si>
+  <si>
+    <t>36 x 60 in / 91 x 152 cm</t>
+  </si>
+  <si>
+    <t>IAC-021</t>
   </si>
   <si>
     <t>Nirakar Chaudhary</t>
@@ -130,13 +166,13 @@
     <t>140 x 85 cm</t>
   </si>
   <si>
-    <t>IAC-014</t>
+    <t>IAC-022</t>
   </si>
   <si>
     <t>153 x 191 cm</t>
   </si>
   <si>
-    <t>IAC-015</t>
+    <t>IAC-023</t>
   </si>
   <si>
     <t>M. D. Ishak</t>
@@ -145,30 +181,6 @@
     <t>Realism</t>
   </si>
   <si>
-    <t>IAC-016</t>
-  </si>
-  <si>
-    <t>IAC-017</t>
-  </si>
-  <si>
-    <t>IAC-018</t>
-  </si>
-  <si>
-    <t>IAC-019</t>
-  </si>
-  <si>
-    <t>IAC-020</t>
-  </si>
-  <si>
-    <t>IAC-021</t>
-  </si>
-  <si>
-    <t>IAC-022</t>
-  </si>
-  <si>
-    <t>IAC-023</t>
-  </si>
-  <si>
     <t>IAC-024</t>
   </si>
   <si>
@@ -229,9 +241,24 @@
     <t>IAC-043</t>
   </si>
   <si>
+    <t>Ashok Rathod</t>
+  </si>
+  <si>
+    <t>Contemporary</t>
+  </si>
+  <si>
+    <t>Nandi</t>
+  </si>
+  <si>
+    <t>24 x 24 in</t>
+  </si>
+  <si>
     <t>IAC-044</t>
   </si>
   <si>
+    <t>36 x 60 in</t>
+  </si>
+  <si>
     <t>IAC-045</t>
   </si>
   <si>
@@ -241,9 +268,15 @@
     <t>IAC-047</t>
   </si>
   <si>
+    <t>48 x 72 in</t>
+  </si>
+  <si>
     <t>IAC-048</t>
   </si>
   <si>
+    <t>Gopal Naskar</t>
+  </si>
+  <si>
     <t>IAC-049</t>
   </si>
   <si>
@@ -256,6 +289,12 @@
     <t>IAC-052</t>
   </si>
   <si>
+    <t>Umendra P. Singh</t>
+  </si>
+  <si>
+    <t>Oil on Canvas</t>
+  </si>
+  <si>
     <t>IAC-053</t>
   </si>
   <si>
@@ -268,6 +307,18 @@
     <t>IAC-056</t>
   </si>
   <si>
+    <t>M. Salim</t>
+  </si>
+  <si>
+    <t>Impressionism</t>
+  </si>
+  <si>
+    <t>Landscape</t>
+  </si>
+  <si>
+    <t>Mix Medium</t>
+  </si>
+  <si>
     <t>IAC-057</t>
   </si>
   <si>
@@ -280,6 +331,9 @@
     <t>IAC-060</t>
   </si>
   <si>
+    <t>Santosh Kumar Shandilya</t>
+  </si>
+  <si>
     <t>IAC-061</t>
   </si>
   <si>
@@ -304,18 +358,48 @@
     <t>IAC-068</t>
   </si>
   <si>
+    <t>Swapon Roy</t>
+  </si>
+  <si>
+    <t>Front the Door</t>
+  </si>
+  <si>
+    <t>36 x 48 in</t>
+  </si>
+  <si>
+    <t>Acrylic and oil on canvas</t>
+  </si>
+  <si>
     <t>IAC-069</t>
   </si>
   <si>
+    <t>Eternal Peace</t>
+  </si>
+  <si>
+    <t>30 x 40 in</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
     <t>IAC-070</t>
   </si>
   <si>
+    <t>Another Way</t>
+  </si>
+  <si>
     <t>IAC-071</t>
   </si>
   <si>
+    <t>At Nalanda</t>
+  </si>
+  <si>
     <t>IAC-072</t>
   </si>
   <si>
+    <t>Unknown Artist</t>
+  </si>
+  <si>
     <t>IAC-073</t>
   </si>
   <si>
@@ -346,22 +430,13 @@
     <t>IAC-082</t>
   </si>
   <si>
-    <t>Ashok Rathod</t>
-  </si>
-  <si>
-    <t>Contemporary</t>
-  </si>
-  <si>
-    <t>Nandi</t>
-  </si>
-  <si>
-    <t>24 x 24 in</t>
-  </si>
-  <si>
     <t>IAC-083</t>
   </si>
   <si>
-    <t>36 x 60 in</t>
+    <t>Folk &amp; Tribal Masters</t>
+  </si>
+  <si>
+    <t>Traditional Folk Art</t>
   </si>
   <si>
     <t>IAC-084</t>
@@ -373,15 +448,9 @@
     <t>IAC-086</t>
   </si>
   <si>
-    <t>48 x 72 in</t>
-  </si>
-  <si>
     <t>IAC-087</t>
   </si>
   <si>
-    <t>Gopal Naskar</t>
-  </si>
-  <si>
     <t>IAC-088</t>
   </si>
   <si>
@@ -394,12 +463,6 @@
     <t>IAC-091</t>
   </si>
   <si>
-    <t>Umendra P. Singh</t>
-  </si>
-  <si>
-    <t>Oil on Canvas</t>
-  </si>
-  <si>
     <t>IAC-092</t>
   </si>
   <si>
@@ -412,18 +475,6 @@
     <t>IAC-095</t>
   </si>
   <si>
-    <t>M. Salim</t>
-  </si>
-  <si>
-    <t>Impressionism</t>
-  </si>
-  <si>
-    <t>Landscape</t>
-  </si>
-  <si>
-    <t>Mix Medium</t>
-  </si>
-  <si>
     <t>IAC-096</t>
   </si>
   <si>
@@ -436,12 +487,6 @@
     <t>IAC-099</t>
   </si>
   <si>
-    <t>Folk &amp; Tribal Masters</t>
-  </si>
-  <si>
-    <t>Traditional Folk Art</t>
-  </si>
-  <si>
     <t>IAC-100</t>
   </si>
   <si>
@@ -589,82 +634,34 @@
     <t>IAC-148</t>
   </si>
   <si>
+    <t>N. K. Mishra</t>
+  </si>
+  <si>
+    <t>21.5 x 15 in</t>
+  </si>
+  <si>
+    <t>Water colour and gouache on paper</t>
+  </si>
+  <si>
     <t>IAC-149</t>
   </si>
   <si>
+    <t>Parvati and Ganesha</t>
+  </si>
+  <si>
+    <t>13.2 x 7.1 in</t>
+  </si>
+  <si>
     <t>IAC-150</t>
   </si>
   <si>
+    <t>Ganesh</t>
+  </si>
+  <si>
+    <t>12.5 x 8.5 in</t>
+  </si>
+  <si>
     <t>IAC-151</t>
-  </si>
-  <si>
-    <t>IAC-152</t>
-  </si>
-  <si>
-    <t>IAC-153</t>
-  </si>
-  <si>
-    <t>IAC-154</t>
-  </si>
-  <si>
-    <t>IAC-155</t>
-  </si>
-  <si>
-    <t>IAC-156</t>
-  </si>
-  <si>
-    <t>IAC-157</t>
-  </si>
-  <si>
-    <t>IAC-158</t>
-  </si>
-  <si>
-    <t>IAC-159</t>
-  </si>
-  <si>
-    <t>IAC-160</t>
-  </si>
-  <si>
-    <t>IAC-161</t>
-  </si>
-  <si>
-    <t>IAC-162</t>
-  </si>
-  <si>
-    <t>IAC-163</t>
-  </si>
-  <si>
-    <t>IAC-164</t>
-  </si>
-  <si>
-    <t>N. K. Mishra</t>
-  </si>
-  <si>
-    <t>21.5 x 15 in</t>
-  </si>
-  <si>
-    <t>Water colour and gouache on paper</t>
-  </si>
-  <si>
-    <t>IAC-165</t>
-  </si>
-  <si>
-    <t>Parvati and Ganesha</t>
-  </si>
-  <si>
-    <t>13.2 x 7.1 in</t>
-  </si>
-  <si>
-    <t>IAC-166</t>
-  </si>
-  <si>
-    <t>Ganesh</t>
-  </si>
-  <si>
-    <t>12.5 x 8.5 in</t>
-  </si>
-  <si>
-    <t>IAC-167</t>
   </si>
   <si>
     <t>Hanuman</t>
@@ -1075,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1281,16 +1278,16 @@
         <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>14</v>
@@ -1298,7 +1295,7 @@
     </row>
     <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
@@ -1307,16 +1304,16 @@
         <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>14</v>
@@ -1324,25 +1321,25 @@
     </row>
     <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>14</v>
@@ -1350,25 +1347,25 @@
     </row>
     <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>14</v>
@@ -1376,25 +1373,25 @@
     </row>
     <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>14</v>
@@ -1402,25 +1399,25 @@
     </row>
     <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>14</v>
@@ -1428,25 +1425,25 @@
     </row>
     <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>14</v>
@@ -1454,25 +1451,25 @@
     </row>
     <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>14</v>
@@ -1480,25 +1477,25 @@
     </row>
     <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>14</v>
@@ -1506,25 +1503,25 @@
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>14</v>
@@ -1532,25 +1529,25 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>14</v>
@@ -1558,25 +1555,25 @@
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="F19" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>14</v>
@@ -1584,22 +1581,22 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>11</v>
@@ -1610,25 +1607,25 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>14</v>
@@ -1636,22 +1633,22 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>11</v>
@@ -1662,22 +1659,22 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>11</v>
@@ -1688,13 +1685,13 @@
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>11</v>
@@ -1714,13 +1711,13 @@
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>11</v>
@@ -1740,13 +1737,13 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>11</v>
@@ -1766,13 +1763,13 @@
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="C27" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
@@ -1792,13 +1789,13 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>11</v>
@@ -1818,13 +1815,13 @@
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>11</v>
@@ -1844,13 +1841,13 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>11</v>
@@ -1870,13 +1867,13 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>11</v>
@@ -1896,13 +1893,13 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>11</v>
@@ -1922,13 +1919,13 @@
     </row>
     <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>11</v>
@@ -1948,13 +1945,13 @@
     </row>
     <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>11</v>
@@ -1974,13 +1971,13 @@
     </row>
     <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>11</v>
@@ -2000,13 +1997,13 @@
     </row>
     <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>11</v>
@@ -2026,13 +2023,13 @@
     </row>
     <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>11</v>
@@ -2052,13 +2049,13 @@
     </row>
     <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>11</v>
@@ -2078,13 +2075,13 @@
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>11</v>
@@ -2104,13 +2101,13 @@
     </row>
     <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>11</v>
@@ -2130,13 +2127,13 @@
     </row>
     <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>11</v>
@@ -2156,13 +2153,13 @@
     </row>
     <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>11</v>
@@ -2182,13 +2179,13 @@
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>11</v>
@@ -2208,22 +2205,22 @@
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>11</v>
@@ -2234,22 +2231,22 @@
     </row>
     <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>11</v>
@@ -2260,22 +2257,22 @@
     </row>
     <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>11</v>
@@ -2286,22 +2283,22 @@
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>11</v>
@@ -2312,22 +2309,22 @@
     </row>
     <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>11</v>
@@ -2338,22 +2335,22 @@
     </row>
     <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>11</v>
@@ -2364,22 +2361,22 @@
     </row>
     <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="D50" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>11</v>
@@ -2390,22 +2387,22 @@
     </row>
     <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>11</v>
@@ -2416,22 +2413,22 @@
     </row>
     <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="F52" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>11</v>
@@ -2442,13 +2439,13 @@
     </row>
     <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>11</v>
@@ -2457,7 +2454,7 @@
         <v>11</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>11</v>
@@ -2468,13 +2465,13 @@
     </row>
     <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>11</v>
@@ -2483,7 +2480,7 @@
         <v>11</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>11</v>
@@ -2494,13 +2491,13 @@
     </row>
     <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>11</v>
@@ -2509,7 +2506,7 @@
         <v>11</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>11</v>
@@ -2520,13 +2517,13 @@
     </row>
     <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>11</v>
@@ -2535,7 +2532,7 @@
         <v>11</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>11</v>
@@ -2546,22 +2543,22 @@
     </row>
     <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>11</v>
@@ -2572,22 +2569,22 @@
     </row>
     <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>11</v>
@@ -2598,22 +2595,22 @@
     </row>
     <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>11</v>
@@ -2624,22 +2621,22 @@
     </row>
     <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>11</v>
@@ -2650,13 +2647,13 @@
     </row>
     <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>11</v>
@@ -2676,13 +2673,13 @@
     </row>
     <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>11</v>
@@ -2702,13 +2699,13 @@
     </row>
     <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>11</v>
@@ -2728,13 +2725,13 @@
     </row>
     <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>11</v>
@@ -2754,13 +2751,13 @@
     </row>
     <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>11</v>
@@ -2780,13 +2777,13 @@
     </row>
     <row r="66" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>11</v>
@@ -2806,13 +2803,13 @@
     </row>
     <row r="67" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>11</v>
@@ -2832,13 +2829,13 @@
     </row>
     <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>11</v>
@@ -2858,22 +2855,22 @@
     </row>
     <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>11</v>
+        <v>117</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>11</v>
@@ -2884,25 +2881,25 @@
     </row>
     <row r="70" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>11</v>
+        <v>121</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="H70" s="4" t="s">
         <v>14</v>
@@ -2910,22 +2907,22 @@
     </row>
     <row r="71" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>11</v>
+        <v>124</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>11</v>
+        <v>121</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>11</v>
@@ -2936,22 +2933,22 @@
     </row>
     <row r="72" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>11</v>
+        <v>126</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>11</v>
+        <v>117</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>11</v>
@@ -2962,13 +2959,13 @@
     </row>
     <row r="73" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>11</v>
@@ -2988,13 +2985,13 @@
     </row>
     <row r="74" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>11</v>
@@ -3014,13 +3011,13 @@
     </row>
     <row r="75" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>11</v>
@@ -3040,13 +3037,13 @@
     </row>
     <row r="76" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>11</v>
@@ -3066,13 +3063,13 @@
     </row>
     <row r="77" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>11</v>
@@ -3092,13 +3089,13 @@
     </row>
     <row r="78" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>105</v>
+        <v>133</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>11</v>
@@ -3118,13 +3115,13 @@
     </row>
     <row r="79" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>106</v>
+        <v>134</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>11</v>
@@ -3144,13 +3141,13 @@
     </row>
     <row r="80" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>11</v>
@@ -3170,13 +3167,13 @@
     </row>
     <row r="81" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>108</v>
+        <v>136</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>11</v>
@@ -3196,13 +3193,13 @@
     </row>
     <row r="82" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>11</v>
@@ -3222,22 +3219,22 @@
     </row>
     <row r="83" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>11</v>
@@ -3248,22 +3245,22 @@
     </row>
     <row r="84" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>11</v>
@@ -3274,22 +3271,22 @@
     </row>
     <row r="85" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>11</v>
@@ -3300,22 +3297,22 @@
     </row>
     <row r="86" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>11</v>
@@ -3326,22 +3323,22 @@
     </row>
     <row r="87" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>120</v>
+        <v>11</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>11</v>
@@ -3352,22 +3349,22 @@
     </row>
     <row r="88" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>11</v>
@@ -3378,22 +3375,22 @@
     </row>
     <row r="89" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>11</v>
@@ -3404,22 +3401,22 @@
     </row>
     <row r="90" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>11</v>
@@ -3430,22 +3427,22 @@
     </row>
     <row r="91" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>11</v>
@@ -3456,13 +3453,13 @@
     </row>
     <row r="92" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>11</v>
@@ -3471,7 +3468,7 @@
         <v>11</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>11</v>
@@ -3482,13 +3479,13 @@
     </row>
     <row r="93" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>11</v>
@@ -3497,7 +3494,7 @@
         <v>11</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>11</v>
@@ -3508,13 +3505,13 @@
     </row>
     <row r="94" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>11</v>
@@ -3523,7 +3520,7 @@
         <v>11</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>11</v>
@@ -3534,13 +3531,13 @@
     </row>
     <row r="95" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>11</v>
@@ -3549,7 +3546,7 @@
         <v>11</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>11</v>
@@ -3560,22 +3557,22 @@
     </row>
     <row r="96" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>11</v>
@@ -3586,22 +3583,22 @@
     </row>
     <row r="97" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="G97" s="2" t="s">
         <v>11</v>
@@ -3612,22 +3609,22 @@
     </row>
     <row r="98" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="G98" s="2" t="s">
         <v>11</v>
@@ -3638,22 +3635,22 @@
     </row>
     <row r="99" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>135</v>
+        <v>11</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="G99" s="2" t="s">
         <v>11</v>
@@ -3664,13 +3661,13 @@
     </row>
     <row r="100" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>11</v>
@@ -3690,13 +3687,13 @@
     </row>
     <row r="101" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>11</v>
@@ -3716,13 +3713,13 @@
     </row>
     <row r="102" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D102" s="2" t="s">
         <v>11</v>
@@ -3742,13 +3739,13 @@
     </row>
     <row r="103" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D103" s="2" t="s">
         <v>11</v>
@@ -3768,13 +3765,13 @@
     </row>
     <row r="104" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D104" s="2" t="s">
         <v>11</v>
@@ -3794,13 +3791,13 @@
     </row>
     <row r="105" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D105" s="2" t="s">
         <v>11</v>
@@ -3820,13 +3817,13 @@
     </row>
     <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D106" s="2" t="s">
         <v>11</v>
@@ -3846,13 +3843,13 @@
     </row>
     <row r="107" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D107" s="2" t="s">
         <v>11</v>
@@ -3872,13 +3869,13 @@
     </row>
     <row r="108" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>11</v>
@@ -3898,13 +3895,13 @@
     </row>
     <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D109" s="2" t="s">
         <v>11</v>
@@ -3924,13 +3921,13 @@
     </row>
     <row r="110" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D110" s="2" t="s">
         <v>11</v>
@@ -3950,13 +3947,13 @@
     </row>
     <row r="111" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D111" s="2" t="s">
         <v>11</v>
@@ -3976,13 +3973,13 @@
     </row>
     <row r="112" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D112" s="2" t="s">
         <v>11</v>
@@ -4002,13 +3999,13 @@
     </row>
     <row r="113" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D113" s="2" t="s">
         <v>11</v>
@@ -4028,13 +4025,13 @@
     </row>
     <row r="114" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D114" s="2" t="s">
         <v>11</v>
@@ -4054,13 +4051,13 @@
     </row>
     <row r="115" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D115" s="2" t="s">
         <v>11</v>
@@ -4080,13 +4077,13 @@
     </row>
     <row r="116" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D116" s="2" t="s">
         <v>11</v>
@@ -4106,13 +4103,13 @@
     </row>
     <row r="117" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D117" s="2" t="s">
         <v>11</v>
@@ -4132,13 +4129,13 @@
     </row>
     <row r="118" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D118" s="2" t="s">
         <v>11</v>
@@ -4158,13 +4155,13 @@
     </row>
     <row r="119" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D119" s="2" t="s">
         <v>11</v>
@@ -4184,13 +4181,13 @@
     </row>
     <row r="120" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D120" s="2" t="s">
         <v>11</v>
@@ -4210,13 +4207,13 @@
     </row>
     <row r="121" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D121" s="2" t="s">
         <v>11</v>
@@ -4236,13 +4233,13 @@
     </row>
     <row r="122" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D122" s="2" t="s">
         <v>11</v>
@@ -4262,13 +4259,13 @@
     </row>
     <row r="123" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D123" s="2" t="s">
         <v>11</v>
@@ -4288,13 +4285,13 @@
     </row>
     <row r="124" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D124" s="2" t="s">
         <v>11</v>
@@ -4314,13 +4311,13 @@
     </row>
     <row r="125" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D125" s="2" t="s">
         <v>11</v>
@@ -4340,13 +4337,13 @@
     </row>
     <row r="126" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D126" s="2" t="s">
         <v>11</v>
@@ -4366,13 +4363,13 @@
     </row>
     <row r="127" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D127" s="2" t="s">
         <v>11</v>
@@ -4392,13 +4389,13 @@
     </row>
     <row r="128" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D128" s="2" t="s">
         <v>11</v>
@@ -4418,13 +4415,13 @@
     </row>
     <row r="129" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D129" s="2" t="s">
         <v>11</v>
@@ -4444,13 +4441,13 @@
     </row>
     <row r="130" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D130" s="2" t="s">
         <v>11</v>
@@ -4470,13 +4467,13 @@
     </row>
     <row r="131" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D131" s="2" t="s">
         <v>11</v>
@@ -4496,13 +4493,13 @@
     </row>
     <row r="132" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D132" s="2" t="s">
         <v>11</v>
@@ -4522,13 +4519,13 @@
     </row>
     <row r="133" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D133" s="2" t="s">
         <v>11</v>
@@ -4548,13 +4545,13 @@
     </row>
     <row r="134" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D134" s="2" t="s">
         <v>11</v>
@@ -4574,13 +4571,13 @@
     </row>
     <row r="135" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D135" s="2" t="s">
         <v>11</v>
@@ -4600,13 +4597,13 @@
     </row>
     <row r="136" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D136" s="2" t="s">
         <v>11</v>
@@ -4626,13 +4623,13 @@
     </row>
     <row r="137" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D137" s="2" t="s">
         <v>11</v>
@@ -4652,13 +4649,13 @@
     </row>
     <row r="138" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D138" s="2" t="s">
         <v>11</v>
@@ -4678,13 +4675,13 @@
     </row>
     <row r="139" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D139" s="2" t="s">
         <v>11</v>
@@ -4704,13 +4701,13 @@
     </row>
     <row r="140" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D140" s="2" t="s">
         <v>11</v>
@@ -4730,13 +4727,13 @@
     </row>
     <row r="141" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D141" s="2" t="s">
         <v>11</v>
@@ -4756,13 +4753,13 @@
     </row>
     <row r="142" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D142" s="2" t="s">
         <v>11</v>
@@ -4782,13 +4779,13 @@
     </row>
     <row r="143" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D143" s="2" t="s">
         <v>11</v>
@@ -4808,13 +4805,13 @@
     </row>
     <row r="144" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D144" s="2" t="s">
         <v>11</v>
@@ -4834,13 +4831,13 @@
     </row>
     <row r="145" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D145" s="2" t="s">
         <v>11</v>
@@ -4860,13 +4857,13 @@
     </row>
     <row r="146" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D146" s="2" t="s">
         <v>11</v>
@@ -4886,13 +4883,13 @@
     </row>
     <row r="147" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D147" s="2" t="s">
         <v>11</v>
@@ -4912,13 +4909,13 @@
     </row>
     <row r="148" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D148" s="2" t="s">
         <v>11</v>
@@ -4938,22 +4935,22 @@
     </row>
     <row r="149" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="D149" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>11</v>
+        <v>208</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>11</v>
+        <v>209</v>
       </c>
       <c r="G149" s="2" t="s">
         <v>11</v>
@@ -4964,22 +4961,22 @@
     </row>
     <row r="150" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>11</v>
+        <v>211</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>11</v>
+        <v>212</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>11</v>
+        <v>209</v>
       </c>
       <c r="G150" s="2" t="s">
         <v>11</v>
@@ -4990,22 +4987,22 @@
     </row>
     <row r="151" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>11</v>
+        <v>214</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>11</v>
+        <v>215</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>11</v>
+        <v>209</v>
       </c>
       <c r="G151" s="2" t="s">
         <v>11</v>
@@ -5016,22 +5013,22 @@
     </row>
     <row r="152" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>11</v>
+        <v>217</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>11</v>
+        <v>218</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>11</v>
+        <v>209</v>
       </c>
       <c r="G152" s="2" t="s">
         <v>11</v>
@@ -5040,424 +5037,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="153" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="B153" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D153" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E153" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F153" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G153" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H153" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B154" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D154" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F154" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G154" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H154" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="B155" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D155" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E155" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F155" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G155" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H155" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="B156" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D156" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E156" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F156" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G156" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H156" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B157" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D157" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E157" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F157" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G157" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H157" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="158" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="B158" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D158" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E158" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F158" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G158" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H158" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="159" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B159" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C159" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D159" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E159" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F159" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G159" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H159" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="160" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B160" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C160" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F160" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G160" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H160" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B161" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C161" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E161" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F161" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G161" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H161" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="162" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="B162" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C162" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H162" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="163" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B163" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C163" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D163" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E163" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F163" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G163" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H163" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B164" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C164" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E164" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F164" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G164" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H164" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="165" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B165" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C165" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E165" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="F165" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G165" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H165" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B166" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E166" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="F166" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G166" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H166" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="167" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="B167" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C167" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D167" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E167" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="F167" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G167" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H167" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="B168" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C168" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D168" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="E168" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F168" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G168" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H168" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H168"/>
+  <autoFilter ref="A1:H152"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>